<commit_message>
data: fireballvolley range 5 -> 10
</commit_message>
<xml_diff>
--- a/xls/ability.xlsx
+++ b/xls/ability.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
     <workbookView xWindow="750" yWindow="1185" windowWidth="19200" windowHeight="6450" activeTab="3"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="general" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="sword" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="archery" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="fire" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="ice" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="poison" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="support" state="visible" r:id="rId10"/>
-    <sheet sheetId="8" name="enhancement" state="visible" r:id="rId11"/>
+    <sheet name="general" sheetId="1" r:id="rId1"/>
+    <sheet name="sword" sheetId="2" r:id="rId2"/>
+    <sheet name="archery" sheetId="3" r:id="rId3"/>
+    <sheet name="fire" sheetId="4" r:id="rId4"/>
+    <sheet name="ice" sheetId="5" r:id="rId5"/>
+    <sheet name="poison" sheetId="6" r:id="rId6"/>
+    <sheet name="support" sheetId="7" r:id="rId7"/>
+    <sheet name="enhancement" sheetId="8" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -59,11 +59,11 @@
     <t>passive</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"偷竊",
+    <t>"lab":"偷竊",
 "des":"從 NPC 或怪物身上獲取財物。成功率視敏捷而定。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Stealing",
+    <t>"lab":"Stealing",
 "des":"從 NPC 或怪物身上獲取財物。成功率視敏捷而定。"</t>
   </si>
   <si>
@@ -73,11 +73,11 @@
     <t>🗝️</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"開鎖",
+    <t>"lab":"開鎖",
 "des":"破解寶箱或門鎖。解鎖更高難度的鎖具。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Lockpicking",
+    <t>"lab":"Lockpicking",
 "des":"破解寶箱或門鎖。解鎖更高難度的鎖具。"</t>
   </si>
   <si>
@@ -87,11 +87,11 @@
     <t>🔪</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"解剖",
+    <t>"lab":"解剖",
 "des":"分解動物屍體，取得肉類、皮毛與骨頭...等可用素材。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Butcher",
+    <t>"lab":"Butcher",
 "des":"分解動物屍體，取得肉類、皮毛與骨頭...等可用素材。"</t>
   </si>
   <si>
@@ -101,11 +101,11 @@
     <t>👤</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"潛行",
+    <t>"lab":"潛行",
 "des":"進入半透明狀態，大幅降低敵方偵測範圍。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Stealth",
+    <t>"lab":"Stealth",
 "des":"進入半透明狀態，大幅降低敵方偵測範圍。"</t>
   </si>
   <si>
@@ -115,11 +115,11 @@
     <t>💰</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"討價還價",
+    <t>"lab":"討價還價",
 "des":"交易時獲得更好價格。商店售價 -15%，回收價 +15%。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Barter",
+    <t>"lab":"Barter",
 "des":"交易時獲得更好價格。商店售價 -15%，回收價 +15%。"</t>
   </si>
   <si>
@@ -141,11 +141,11 @@
     <t>"hits":[{"pow":1.15,"flat":0}],"range":1,"cd":1,"travel":{"type":"melee"}</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"斬擊",
+    <t>"lab":"斬擊",
 "des":"基本橫劈，對前方弧形範圍造成 115% 傷害。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Slash",
+    <t>"lab":"Slash",
 "des":"基本橫劈，對前方弧形範圍造成 115% 傷害。"</t>
   </si>
   <si>
@@ -158,11 +158,11 @@
     <t>"hits":[{"pow":1.0,"flat":0,"pen":0.2}],"range":1,"cd":1,"travel":{"type":"melee"}</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"刺擊",
+    <t>"lab":"刺擊",
 "des":"直線突刺。無視目標 20% 物理防禦。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Thrust",
+    <t>"lab":"Thrust",
 "des":"直線突刺。無視目標 20% 物理防禦。"</t>
   </si>
   <si>
@@ -178,11 +178,11 @@
     <t>"range":1,"cd":3,"scope":"group","w":3,"h":3,"cast":{},"fx":{}</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"旋風斬",
+    <t>"lab":"旋風斬",
 "des":"旋轉劍身，對周圍範圍{#wh}方格造成多段傷害。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Whirlwind",
+    <t>"lab":"Whirlwind",
 "des":"旋轉劍身，對周圍範圍{#wh}方格造成多段傷害。"</t>
   </si>
   <si>
@@ -195,15 +195,15 @@
     <t>buff</t>
   </si>
   <si>
-    <t xml:space="preserve">{"type":"mod","key":"acc","a":0.1,"reqClass":"sword"},
+    <t>{"type":"mod","key":"acc","a":0.1,"reqClass":"sword"},
 {"type":"mod","key":"atk","m":0.1,"reqClass":"sword"}</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"劍術專家",
+    <t>"lab":"劍術專家",
 "des":"精通劍術。裝備劍類武器時，命中+10%、攻擊力+10%。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Sword Expertise",
+    <t>"lab":"Sword Expertise",
 "des":"Mastery of swordsmanship. +10% accuracy and +10% attack power while wielding a sword."</t>
   </si>
   <si>
@@ -216,15 +216,15 @@
     <t>"swordmastery"</t>
   </si>
   <si>
-    <t xml:space="preserve">{"type":"mod","key":"acc","a":0.15,"reqClass":"sword"},
+    <t>{"type":"mod","key":"acc","a":0.15,"reqClass":"sword"},
 {"type":"mod","key":"atk","m":0.15,"reqClass":"sword"}</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"劍術大師",
+    <t>"lab":"劍術大師",
 "des":"劍術造詣爐火純青。裝備劍類武器時，命中與攻擊力再進一步大幅提升。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Sword Mastery",
+    <t>"lab":"Sword Mastery",
 "des":"Peak swordsmanship. Further boosts accuracy and attack power while wielding a sword."</t>
   </si>
   <si>
@@ -237,11 +237,11 @@
     <t>"hits":[{"pow":2.5,"flat":0}],"range":5,"cd":3,"travel":{"type":"ranged"}</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"狙擊",
+    <t>"lab":"狙擊",
 "des":"瞄準敵人的弱點射擊，造成 250% 的傷害。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Snipe",
+    <t>"lab":"Snipe",
 "des":"瞄準敵人的弱點射擊，造成 250% 的傷害。"</t>
   </si>
   <si>
@@ -251,15 +251,15 @@
     <t>🏹</t>
   </si>
   <si>
-    <t xml:space="preserve">{"type":"mod","key":"acc","a":0.1,"reqClass":"bow"},
+    <t>{"type":"mod","key":"acc","a":0.1,"reqClass":"bow"},
 {"type":"mod","key":"atk","m":0.1,"reqClass":"bow"}</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"弓箭專家",
+    <t>"lab":"弓箭專家",
 "des":"精通弓術。裝備弓類武器時，命中+10%、攻擊力+10%。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Archery Expertise",
+    <t>"lab":"Archery Expertise",
 "des":"Mastery of archery. +10% accuracy and +10% attack power while wielding a bow."</t>
   </si>
   <si>
@@ -272,15 +272,15 @@
     <t>"archeryexpert"</t>
   </si>
   <si>
-    <t xml:space="preserve">{"type":"mod","key":"acc","a":0.15,"reqClass":"bow"},
+    <t>{"type":"mod","key":"acc","a":0.15,"reqClass":"bow"},
 {"type":"mod","key":"atk","m":0.15,"reqClass":"bow"}</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"弓箭大師",
+    <t>"lab":"弓箭大師",
 "des":"弓術造詣爐火純青。裝備弓類武器時，命中與攻擊力再進一步大幅提升。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Archery Mastery",
+    <t>"lab":"Archery Mastery",
 "des":"Peak archery. Further boosts accuracy and attack power while wielding a bow."</t>
   </si>
   <si>
@@ -296,11 +296,11 @@
     <t>{"type":"dot","scope":"target","stage":"hit","elm":"fire","a":-5,"dur":3,"icon":"🔥","id":"burn","stack":3}</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"火球術",
+    <t>"lab":"火球術",
 "des":"投擲火球，造成 {#fmt} 點{#elm}爆炸傷害({#formula})。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Fireball",
+    <t>"lab":"Fireball",
 "des":"投擲火球，造成 {#fmt} 點{#elm}爆炸傷害({#formula})。"</t>
   </si>
   <si>
@@ -316,11 +316,11 @@
     <t>"cd":3,"range":5,"cast":{},"zoneW":5,"zoneH":1,"zoneDur":4,"zoneImg":"🔥","zoneAnim":{"cell":{"size":30,"jitter":3,"scale":[0.85,1.15],"alpha":0.9,"flipX":"random"},"spawn":{"scale":{"from":0,"to":1},"duration":250,"ease":"Back.Out","stagger":70,"from":"center"},"idle":{"scaleX":{"from":0.75,"to":1.25},"scaleY":{"from":0.75,"to":1.25},"y":"-=2","duration":450,"yoyo":true,"repeat":-1,"ease":"Sine.InOut","randDelay":450},"tick":{"scale":{"from":1,"to":1.4},"duration":150,"yoyo":true,"ease":"Quad.Out"},"end":{"alpha":0,"scale":0.3,"duration":350,"ease":"Quad.In"}}</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"火牆術",
+    <t>"lab":"火牆術",
 "des":"召喚{#wh}方格的火焰地帶。對經過者施加持續灼燒。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Fire Wall",
+    <t>"lab":"Fire Wall",
 "des":"召喚{#wh}方格的火焰地帶。對經過者施加持續灼燒。"</t>
   </si>
   <si>
@@ -330,14 +330,11 @@
     <t>"fireball"</t>
   </si>
   <si>
-    <t>"scope":"cone","range":5,"angle":45,"hits":[{"elm":"fire","pow":1.8,"flat":10,"src":"int"}],"cd":5,"travel":{"type":"spell","img":"🔥","size":25,"deg":-90},"fx":{}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"lab":"高級火球術",
+    <t>"lab":"高級火球術",
 "des":"朝指定方向 {#angle}° 扇形、{#range} 格內的每個角色各自發射火球，每發造成 {#fmt} 點{#elm}傷害({#formula})。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Greater Fireball",
+    <t>"lab":"Greater Fireball",
 "des":"Fires a fireball at each character within a {#angle}° cone up to {#range} tiles in the chosen direction, dealing {#fmt} {#elm} damage each ({#formula})."</t>
   </si>
   <si>
@@ -347,18 +344,18 @@
     <t>🌋</t>
   </si>
   <si>
-    <t xml:space="preserve">"fireballvolley",
+    <t>"fireballvolley",
 "firewall"</t>
   </si>
   <si>
     <t>"range":5,"hits":[{"elm":"fire","pow":2.0,"flat":15,"src":"int"}],"cd":4,"scope":"group","w":5,"h":5,"cast":{},"fx":{}</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"燃燒術",
+    <t>"lab":"燃燒術",
 "des":"引爆範圍{#wh}方格內目標身上的灼燒狀態，造成 {#fmt} 點{#elm}瞬間大傷害({#formula})。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Combustion",
+    <t>"lab":"Combustion",
 "des":"引爆範圍{#wh}方格內目標身上的灼燒狀態，造成 {#fmt} 點{#elm}瞬間大傷害({#formula})。"</t>
   </si>
   <si>
@@ -374,11 +371,11 @@
     <t>"hits":[{"elm":"fire","pow":2.5,"flat":20,"src":"int"},{"elm":"phy","pow":2,"flat":10,"src":"int"}],"range":5,"cd":6,"scope":"area","w":7,"h":7,"travel":{"type":"fall","img":"☄️","size":25,"deg":-135,"randomDelay":800},"fx":{"img":"🔥"},"carpet":true</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"流星雨",
+    <t>"lab":"流星雨",
 "des":"大範圍{#wh}方格隕石轟炸，每顆造成 {#fmt0} 點{#elm0}傷害({#formula0})及 {#fmt1} 點{#elm1}傷害({#formula1})，摧毀範圍內一切。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Meteor Shower",
+    <t>"lab":"Meteor Shower",
 "des":"大範圍{#wh}方格隕石轟炸，每顆造成 {#fmt0} 點{#elm0}傷害({#formula0})及 {#fmt1} 點{#elm1}傷害({#formula1})，摧毀範圍內一切。"</t>
   </si>
   <si>
@@ -391,11 +388,11 @@
     <t>"hits":[{"elm":"ice","pow":1.5,"flat":10,"src":"int"}],"range":5,"cd":3</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"冰箭術",
+    <t>"lab":"冰箭術",
 "des":"單體冰錐。造成傷害並減速 30%。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Ice Bolt",
+    <t>"lab":"Ice Bolt",
 "des":"單體冰錐。造成傷害並減速 30%。"</t>
   </si>
   <si>
@@ -405,11 +402,11 @@
     <t>🧊</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"冰牆術",
+    <t>"lab":"冰牆術",
 "des":"召喚可抵擋飛行道具的冰塊物理障礙物。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Ice Wall",
+    <t>"lab":"Ice Wall",
 "des":"召喚可抵擋飛行道具的冰塊物理障礙物。"</t>
   </si>
   <si>
@@ -419,18 +416,18 @@
     <t>🥶</t>
   </si>
   <si>
-    <t xml:space="preserve">"icebolt",
+    <t>"icebolt",
 "icewall"</t>
   </si>
   <si>
     <t>"hits":[{"elm":"ice","pow":2.0,"flat":15,"src":"int"}],"range":5,"cd":4</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"冰封術",
+    <t>"lab":"冰封術",
 "des":"將減速狀態轉為凍結，使敵方完全無法行動 3 秒。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Deep Freeze",
+    <t>"lab":"Deep Freeze",
 "des":"將減速狀態轉為凍結，使敵方完全無法行動 3 秒。"</t>
   </si>
   <si>
@@ -446,11 +443,11 @@
     <t>"hits":[{"elm":"ice","pow":2.5,"flat":20,"src":"int"}],"range":5,"cd":6</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"暴風雪",
+    <t>"lab":"暴風雪",
 "des":"大範圍持續性傷害，並有 10% 機率直接凍結敵人。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Blizzard",
+    <t>"lab":"Blizzard",
 "des":"大範圍持續性傷害，並有 10% 機率直接凍結敵人。"</t>
   </si>
   <si>
@@ -463,7 +460,7 @@
     <t>"hits":[{"elm":"poison","pow":1.5,"flat":10,"src":"int"}],"range":5,"cd":3</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"毒箭術",
+    <t>"lab":"毒箭術",
 "des":"遠程發射毒針，使目標進入每秒扣血的中毒狀態。"</t>
   </si>
   <si>
@@ -473,7 +470,7 @@
     <t>🌫️</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"毒霧術",
+    <t>"lab":"毒霧術",
 "des":"在指定區域散佈致命毒氣。"</t>
   </si>
   <si>
@@ -483,14 +480,14 @@
     <t>🍄</t>
   </si>
   <si>
-    <t xml:space="preserve">"poisondart",
+    <t>"poisondart",
 "poisonmist"</t>
   </si>
   <si>
     <t>"hits":[{"elm":"poison","pow":2.0,"flat":15,"src":"int"}],"range":5,"cd":4</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"毒素引爆",
+    <t>"lab":"毒素引爆",
 "des":"使受毒者爆炸，將毒素噴濺至周圍目標。"</t>
   </si>
   <si>
@@ -503,11 +500,11 @@
     <t>"cd":2</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"治療",
+    <t>"lab":"治療",
 "des":"恢復目標生命值。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Heal",
+    <t>"lab":"Heal",
 "des":"恢復目標生命值。"</t>
   </si>
   <si>
@@ -520,11 +517,11 @@
     <t>"cd":3</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"解毒",
+    <t>"lab":"解毒",
 "des":"清除體內毒素。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Cure",
+    <t>"lab":"Cure",
 "des":"清除體內毒素。"</t>
   </si>
   <si>
@@ -534,11 +531,11 @@
     <t>☀️</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"聖光",
+    <t>"lab":"聖光",
 "des":"移除 1 個負面狀態。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Holy Light",
+    <t>"lab":"Holy Light",
 "des":"移除 1 個負面狀態。"</t>
   </si>
   <si>
@@ -548,18 +545,18 @@
     <t>✨</t>
   </si>
   <si>
-    <t xml:space="preserve">"cure",
+    <t>"cure",
 "holylight"</t>
   </si>
   <si>
     <t>"cd":5</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"淨化",
+    <t>"lab":"淨化",
 "des":"清除體內毒素，移除所有負面狀態。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Purify",
+    <t>"lab":"Purify",
 "des":"清除體內毒素，移除所有負面狀態。"</t>
   </si>
   <si>
@@ -569,11 +566,11 @@
     <t>💪</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"力量增強",
+    <t>"lab":"力量增強",
 "des":"增加力量，可提升近戰傷害。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Strength Boost",
+    <t>"lab":"Strength Boost",
 "des":"增加力量，可提升近戰傷害。"</t>
   </si>
   <si>
@@ -583,11 +580,11 @@
     <t>👟</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"敏捷增強",
+    <t>"lab":"敏捷增強",
 "des":"增加敏捷，可提升閃避。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Agility Boost",
+    <t>"lab":"Agility Boost",
 "des":"增加敏捷，可提升閃避。"</t>
   </si>
   <si>
@@ -597,32 +594,43 @@
     <t>🧠</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"智力增強",
+    <t>"lab":"智力增強",
 "des":"增加智力，可提升法術效果。"</t>
   </si>
   <si>
-    <t xml:space="preserve">"lab":"Intelligence Boost",
+    <t>"lab":"Intelligence Boost",
 "des":"增加智力，可提升法術效果。"</t>
+  </si>
+  <si>
+    <t>"scope":"cone","range":10,"angle":45,"hits":[{"elm":"fire","pow":1.8,"flat":10,"src":"int"}],"cd":5,"travel":{"type":"spell","img":"🔥","size":25,"deg":-90},"fx":{}</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="3">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="新細明體"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="微軟正黑體 Light"/>
+      <family val="2"/>
       <charset val="136"/>
-      <color theme="1"/>
-      <family val="2"/>
-      <sz val="12"/>
-      <name val="微軟正黑體 Light"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="新細明體"/>
+      <family val="3"/>
+      <charset val="136"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -655,7 +663,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="一般" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -954,9 +962,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.85546875" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="12.5703125" style="1" customWidth="1"/>
     <col min="2" max="2" width="9.28515625" style="1" customWidth="1"/>
@@ -966,10 +974,11 @@
     <col min="7" max="7" width="14.85546875" style="1" customWidth="1"/>
     <col min="8" max="8" width="64.140625" style="1" customWidth="1"/>
     <col min="9" max="9" width="67.28515625" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.85546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="8.85546875" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -998,7 +1007,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="31.5" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
@@ -1019,7 +1028,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="31.5" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
@@ -1032,7 +1041,6 @@
       <c r="D3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="1"/>
       <c r="H3" s="2" t="s">
         <v>16</v>
       </c>
@@ -1040,7 +1048,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="31.5" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>18</v>
       </c>
@@ -1054,7 +1062,6 @@
         <v>18</v>
       </c>
       <c r="E4" s="2"/>
-      <c r="G4" s="1"/>
       <c r="H4" s="2" t="s">
         <v>20</v>
       </c>
@@ -1062,7 +1069,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="31.5" customHeight="1">
       <c r="A5" s="1" t="s">
         <v>22</v>
       </c>
@@ -1072,7 +1079,6 @@
       <c r="C5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G5" s="1"/>
       <c r="H5" s="2" t="s">
         <v>24</v>
       </c>
@@ -1080,7 +1086,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="31.5" customHeight="1">
       <c r="A6" s="1" t="s">
         <v>26</v>
       </c>
@@ -1098,25 +1104,25 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9">
       <c r="H7" s="2"/>
     </row>
-    <row r="13" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9">
       <c r="F13" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G13" s="1"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I6"/>
-  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.85546875" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="12.42578125" style="1" customWidth="1"/>
     <col min="2" max="4" width="8.85546875" style="1" customWidth="1"/>
@@ -1124,10 +1130,11 @@
     <col min="6" max="6" width="14.7109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="11.42578125" style="1" customWidth="1"/>
     <col min="8" max="9" width="66.42578125" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.85546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="8.85546875" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1156,7 +1163,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="31.5" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>31</v>
       </c>
@@ -1172,7 +1179,6 @@
       <c r="F2" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="G2" s="1"/>
       <c r="H2" s="2" t="s">
         <v>36</v>
       </c>
@@ -1180,7 +1186,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="31.5" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>38</v>
       </c>
@@ -1196,7 +1202,6 @@
       <c r="F3" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="G3" s="1"/>
       <c r="H3" s="2" t="s">
         <v>41</v>
       </c>
@@ -1204,7 +1209,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="31.5" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>43</v>
       </c>
@@ -1223,7 +1228,6 @@
       <c r="F4" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="G4" s="1"/>
       <c r="H4" s="2" t="s">
         <v>47</v>
       </c>
@@ -1231,7 +1235,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="31.5" customHeight="1">
       <c r="A5" s="1" t="s">
         <v>49</v>
       </c>
@@ -1254,7 +1258,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="6" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="31.5" customHeight="1">
       <c r="A6" s="1" t="s">
         <v>55</v>
       </c>
@@ -1281,25 +1285,27 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="200" verticalDpi="200"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I4"/>
-  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.85546875" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="12.42578125" style="1" customWidth="1"/>
     <col min="2" max="5" width="8.85546875" style="1" customWidth="1"/>
     <col min="6" max="6" width="14.7109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="11.42578125" style="1" customWidth="1"/>
     <col min="8" max="9" width="66.42578125" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.85546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="8.85546875" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1328,7 +1334,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="31.5" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>61</v>
       </c>
@@ -1344,7 +1350,6 @@
       <c r="F2" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="G2" s="1"/>
       <c r="H2" s="2" t="s">
         <v>64</v>
       </c>
@@ -1352,7 +1357,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="3" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="31.5" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>66</v>
       </c>
@@ -1375,7 +1380,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="4" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="31.5" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>71</v>
       </c>
@@ -1402,27 +1407,29 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="200" verticalDpi="200"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I14"/>
-  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.85546875" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="18.42578125" style="1" customWidth="1"/>
     <col min="2" max="2" width="9.28515625" style="1" customWidth="1"/>
     <col min="3" max="4" width="10.140625" style="1" customWidth="1"/>
     <col min="5" max="5" width="18.28515625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="101" style="2" customWidth="1"/>
-    <col min="7" max="7" width="14.85546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="101.42578125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="41.5703125" style="1" customWidth="1"/>
     <col min="8" max="9" width="70" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.85546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="8.85546875" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1451,7 +1458,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="31.5" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>77</v>
       </c>
@@ -1477,7 +1484,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="3" ht="105" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="105" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>83</v>
       </c>
@@ -1503,7 +1510,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="31.5" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>89</v>
       </c>
@@ -1520,24 +1527,24 @@
         <v>90</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>91</v>
+        <v>170</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>80</v>
       </c>
       <c r="H4" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="I4" s="2" t="s">
+    </row>
+    <row r="5" spans="1:9" ht="31.5" customHeight="1">
+      <c r="A5" s="1" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="5" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>95</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>33</v>
@@ -1546,27 +1553,27 @@
         <v>34</v>
       </c>
       <c r="E5" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>96</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>97</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>80</v>
       </c>
       <c r="H5" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="I5" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="I5" s="2" t="s">
+    </row>
+    <row r="6" spans="1:9" ht="31.5" customHeight="1">
+      <c r="A6" s="1" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="6" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="B6" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>101</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>33</v>
@@ -1575,41 +1582,41 @@
         <v>34</v>
       </c>
       <c r="E6" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>80</v>
       </c>
       <c r="H6" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="I6" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="I6" s="2" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="8" spans="8:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:9">
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
     </row>
-    <row r="14" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9">
       <c r="F14" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G14" s="1"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.85546875" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="18.42578125" style="1" customWidth="1"/>
     <col min="2" max="2" width="9.28515625" style="1" customWidth="1"/>
@@ -1618,10 +1625,11 @@
     <col min="6" max="6" width="14.140625" style="2" customWidth="1"/>
     <col min="7" max="7" width="14.85546875" style="1" customWidth="1"/>
     <col min="8" max="9" width="70" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.85546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="8.85546875" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1650,12 +1658,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="31.5" customHeight="1">
       <c r="A2" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>107</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>33</v>
@@ -1664,22 +1672,22 @@
         <v>34</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="I2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:9" ht="31.5" customHeight="1">
+      <c r="A3" s="1" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="3" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="B3" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>112</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>33</v>
@@ -1688,22 +1696,21 @@
         <v>34</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="G3" s="1"/>
+        <v>107</v>
+      </c>
       <c r="H3" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="I3" s="2" t="s">
+    </row>
+    <row r="4" spans="1:9" ht="31.5" customHeight="1">
+      <c r="A4" s="1" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="4" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>116</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>33</v>
@@ -1712,25 +1719,24 @@
         <v>34</v>
       </c>
       <c r="E4" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="2" t="s">
+      <c r="I4" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="I4" s="2" t="s">
+    </row>
+    <row r="5" spans="1:9" ht="31.5" customHeight="1">
+      <c r="A5" s="1" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="5" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="B5" t="s">
         <v>121</v>
-      </c>
-      <c r="B5" t="s">
-        <v>122</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>33</v>
@@ -1739,43 +1745,42 @@
         <v>34</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="G5" s="1"/>
-      <c r="H5" s="2" t="s">
+      <c r="I5" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="I5" s="2" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="6" spans="7:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:9">
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
     </row>
-    <row r="7" spans="8:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9">
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
     </row>
-    <row r="13" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9">
       <c r="F13" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G13" s="1"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.85546875" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="18.42578125" style="1" customWidth="1"/>
     <col min="2" max="2" width="9.28515625" style="1" customWidth="1"/>
@@ -1785,10 +1790,11 @@
     <col min="7" max="7" width="14.85546875" style="1" customWidth="1"/>
     <col min="8" max="8" width="61" style="1" customWidth="1"/>
     <col min="9" max="9" width="70" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.85546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="8.85546875" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1817,12 +1823,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="31.5" customHeight="1">
       <c r="A2" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>127</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>128</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>33</v>
@@ -1831,22 +1837,22 @@
         <v>34</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="31.5" customHeight="1">
+      <c r="A3" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="I2" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="3" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="B3" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>132</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>33</v>
@@ -1855,22 +1861,21 @@
         <v>34</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="G3" s="1"/>
+        <v>128</v>
+      </c>
       <c r="H3" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="31.5" customHeight="1">
+      <c r="A4" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="I3" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="4" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>134</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>135</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>33</v>
@@ -1879,49 +1884,48 @@
         <v>34</v>
       </c>
       <c r="E4" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="2" t="s">
-        <v>138</v>
-      </c>
       <c r="I4" s="2" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="5" ht="16.5" customHeight="1" spans="6:9" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="16.5" customHeight="1">
       <c r="F5" s="1"/>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
     </row>
-    <row r="6" spans="7:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9">
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
     </row>
-    <row r="7" spans="8:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9">
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
     </row>
-    <row r="13" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9">
       <c r="F13" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G13" s="1"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.85546875" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="18.42578125" style="1" customWidth="1"/>
     <col min="2" max="2" width="9.28515625" style="1" customWidth="1"/>
@@ -1931,10 +1935,11 @@
     <col min="7" max="7" width="14.85546875" style="1" customWidth="1"/>
     <col min="8" max="8" width="48.42578125" style="1" customWidth="1"/>
     <col min="9" max="9" width="70" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.85546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="8.85546875" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1963,129 +1968,126 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="31.5" customHeight="1">
       <c r="A2" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>139</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>140</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>33</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="I2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:9" ht="31.5" customHeight="1">
+      <c r="A3" s="1" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="3" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="B3" s="1" t="s">
         <v>144</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>145</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>33</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="G3" s="1"/>
-      <c r="H3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="I3" s="2" t="s">
+    </row>
+    <row r="4" spans="1:9" ht="31.5" customHeight="1">
+      <c r="A4" s="1" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="4" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>149</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>150</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>33</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="G4" s="1"/>
+        <v>145</v>
+      </c>
       <c r="H4" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="I4" s="2" t="s">
+    </row>
+    <row r="5" spans="1:9" ht="31.5" customHeight="1">
+      <c r="A5" s="1" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="5" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>154</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>33</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E5" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="G5" s="1"/>
-      <c r="H5" s="2" t="s">
+      <c r="I5" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="I5" s="2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="6" spans="7:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:9">
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
     </row>
-    <row r="7" spans="8:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9">
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
     </row>
-    <row r="13" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9">
       <c r="F13" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G13" s="1"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I12"/>
-  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.85546875" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="23.85546875" style="1" customWidth="1"/>
     <col min="2" max="2" width="9.28515625" style="1" customWidth="1"/>
@@ -2094,10 +2096,11 @@
     <col min="6" max="6" width="14.140625" style="2" customWidth="1"/>
     <col min="7" max="7" width="14.85546875" style="1" customWidth="1"/>
     <col min="8" max="9" width="46" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.85546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="8.85546875" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2126,12 +2129,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="31.5" customHeight="1">
       <c r="A2" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>159</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>160</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>33</v>
@@ -2141,18 +2144,18 @@
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="I2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:9" ht="31.5" customHeight="1">
+      <c r="A3" s="1" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="3" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="B3" s="1" t="s">
         <v>163</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>164</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>33</v>
@@ -2160,20 +2163,19 @@
       <c r="D3" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="G3" s="1"/>
       <c r="H3" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="I3" s="2" t="s">
+    </row>
+    <row r="4" spans="1:9" ht="31.5" customHeight="1">
+      <c r="A4" s="1" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="4" ht="31.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>168</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>33</v>
@@ -2182,31 +2184,30 @@
         <v>51</v>
       </c>
       <c r="E4" s="2"/>
-      <c r="G4" s="1"/>
       <c r="H4" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="5" spans="7:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:9">
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
     </row>
-    <row r="6" spans="8:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9">
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
     </row>
-    <row r="12" spans="6:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9">
       <c r="F12" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G12" s="1"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: sword 技能 des 改用 token：slash/dash 改 {#fmt}/{#elm}/{#formula}、dash 擊退格數用 {#knock}；swordmastery des 拿掉數字(交給 mods 行顯示)；slash us 補英文
</commit_message>
<xml_diff>
--- a/xls/ability.xlsx
+++ b/xls/ability.xlsx
@@ -142,11 +142,11 @@
   </si>
   <si>
     <t xml:space="preserve">"lab":"斬擊",
-"des":"基本橫劈，對前方弧形範圍造成 115% 傷害。"</t>
+"des":"基本橫劈，對前方弧形範圍造成 {#fmt} 點{#elm}傷害。{#formula}"</t>
   </si>
   <si>
     <t xml:space="preserve">"lab":"Slash",
-"des":"基本橫劈，對前方弧形範圍造成 115% 傷害。"</t>
+"des":"A basic horizontal cut, dealing {#fmt} {#elm} damage in an arc ahead.{#formula}"</t>
   </si>
   <si>
     <t>dash</t>
@@ -159,11 +159,11 @@
   </si>
   <si>
     <t xml:space="preserve">"lab":"衝刺",
-"des":"衝向敵人，造成 1.5 倍傷害並擊退 1 格。"</t>
+"des":"衝向敵人，造成 {#fmt} 點{#elm}傷害並擊退 {#knock} 格。{#formula}"</t>
   </si>
   <si>
     <t xml:space="preserve">"lab":"Dash",
-"des":"Dash to an enemy, dealing 1.5x damage and knocking it back 1 tile."</t>
+"des":"Dash to an enemy, dealing {#fmt} {#elm} damage and knocking it back {#knock} tile(s).{#formula}"</t>
   </si>
   <si>
     <t>whirlwind</t>
@@ -200,11 +200,11 @@
   </si>
   <si>
     <t xml:space="preserve">"lab":"劍術專家",
-"des":"精通劍術。裝備劍類武器時，命中+10%、攻擊力+10%。"</t>
+"des":"精通劍術。裝備劍類武器時，提升命中與攻擊力。"</t>
   </si>
   <si>
     <t xml:space="preserve">"lab":"Sword Expertise",
-"des":"Mastery of swordsmanship. +10% accuracy and +10% attack power while wielding a sword."</t>
+"des":"Mastery of swordsmanship. Boosts accuracy and attack power while wielding a sword."</t>
   </si>
   <si>
     <t>swordmaster</t>

</xml_diff>

<commit_message>
feat: snipe des 改用 {#fmt}/{#elm}/{#formula} 並補英文；archeryexpert des 拿掉數字(交給 mods 行顯示)
</commit_message>
<xml_diff>
--- a/xls/ability.xlsx
+++ b/xls/ability.xlsx
@@ -238,11 +238,11 @@
   </si>
   <si>
     <t xml:space="preserve">"lab":"狙擊",
-"des":"瞄準敵人的弱點射擊，造成 250% 的傷害。"</t>
+"des":"瞄準敵人的弱點射擊，造成 {#fmt} 點{#elm}傷害。{#formula}"</t>
   </si>
   <si>
     <t xml:space="preserve">"lab":"Snipe",
-"des":"瞄準敵人的弱點射擊，造成 250% 的傷害。"</t>
+"des":"Aims at an enemy's weak spot, dealing {#fmt} {#elm} damage.{#formula}"</t>
   </si>
   <si>
     <t>archeryexpert</t>
@@ -256,11 +256,11 @@
   </si>
   <si>
     <t xml:space="preserve">"lab":"弓箭專家",
-"des":"精通弓術。裝備弓類武器時，命中+10%、攻擊力+10%。"</t>
+"des":"精通弓術。裝備弓類武器時，提升命中與攻擊力。"</t>
   </si>
   <si>
     <t xml:space="preserve">"lab":"Archery Expertise",
-"des":"Mastery of archery. +10% accuracy and +10% attack power while wielding a bow."</t>
+"des":"Mastery of archery. Boosts accuracy and attack power while wielding a bow."</t>
   </si>
   <si>
     <t>archerymaster</t>

</xml_diff>

<commit_message>
refactor: i18n 第 1 階段：識別字 ASCII 化
- quality 改名：好感→favor、討伐令→bandit_hunt(.kills)、狼患→wolf(.kills)、狼皮生意→pelt_trade、殺.*→kill.*；thread id 跟著改
- spawn 群組 @狼群/@盜賊 → @wolves/@bandits（story.xlsx + m_03x05.json）
- scripts/story.js 檢查 quality/thread/storylet/節點/spawn 名稱必須是 ASCII
- 語系代碼 tw/us → zh-TW/en：xlsx 語言欄標頭改名、設定預設值、讀到舊設定自動轉換
- 測試與 story-architecture.md 同步改名

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/xls/ability.xlsx
+++ b/xls/ability.xlsx
@@ -44,10 +44,10 @@
     <t>effects</t>
   </si>
   <si>
-    <t>tw</t>
-  </si>
-  <si>
-    <t>us</t>
+    <t>zh-TW</t>
+  </si>
+  <si>
+    <t>en</t>
   </si>
   <si>
     <t>steal</t>

</xml_diff>